<commit_message>
Mã VV Xăng E10
</commit_message>
<xml_diff>
--- a/Data/DSKH.xlsx
+++ b/Data/DSKH.xlsx
@@ -1,42 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_BB\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E999CB7D-DDB7-45D1-BCE9-EE1B15DE5FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{438379BF-7DA0-4C73-9210-9421362CC032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8B3CD886-8DDF-4B85-B510-D025734B72F1}"/>
   </bookViews>
   <sheets>
     <sheet name="DSKH" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1845" uniqueCount="1811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1882" uniqueCount="1834">
   <si>
     <t>Tên khách Hàng</t>
   </si>
@@ -5469,6 +5458,75 @@
   </si>
   <si>
     <t>0700522428</t>
+  </si>
+  <si>
+    <t>Công ty CP cơ khí nông nghiệp Nam Trực</t>
+  </si>
+  <si>
+    <t>CHI NHÁNH CÔNG TY TNHH MTV BCA – THĂNG LONG – XÍ NGHIỆP KINH DOANH XĂNG DẦU</t>
+  </si>
+  <si>
+    <t>Doanh nghiệp tư nhân xăng dầu Quang Huy Hải Sơn</t>
+  </si>
+  <si>
+    <t>Công ty TNHH xây dựng &amp; thương mại Hưng Thịnh</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH ĐẦU TƯ PHÁT TRIỂN THÁI AN GROUP</t>
+  </si>
+  <si>
+    <t>Công ty cổ phần đầu tư thương mại Minh Hiếu</t>
+  </si>
+  <si>
+    <t>Công ty TNHH xăng dầu Phú Sơn</t>
+  </si>
+  <si>
+    <t>0600280285</t>
+  </si>
+  <si>
+    <t>0100110856-016</t>
+  </si>
+  <si>
+    <t>0601037290</t>
+  </si>
+  <si>
+    <t>0700893091</t>
+  </si>
+  <si>
+    <t>0600994843</t>
+  </si>
+  <si>
+    <t>0600418790</t>
+  </si>
+  <si>
+    <t>1000333018</t>
+  </si>
+  <si>
+    <t>TN0146</t>
+  </si>
+  <si>
+    <t>TN1675</t>
+  </si>
+  <si>
+    <t>ND0003</t>
+  </si>
+  <si>
+    <t>TN1669</t>
+  </si>
+  <si>
+    <t>TN1679</t>
+  </si>
+  <si>
+    <t>MHIEU</t>
+  </si>
+  <si>
+    <t>TN1668</t>
+  </si>
+  <si>
+    <t>Doanh nghiệp tư nhân Minh Nghĩa</t>
+  </si>
+  <si>
+    <t>Công ty TNHH MTV Hiền Thịnh Vượng</t>
   </si>
 </sst>
 </file>
@@ -5942,13 +6000,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E1E6901-43DC-437F-91F6-DDF1071BC387}">
-  <dimension ref="A1:C615"/>
+  <dimension ref="A1:I627"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="11.25" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="82.5703125" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="8.85546875" style="3"/>
+    <col min="4" max="7" width="8.85546875" style="3"/>
+    <col min="8" max="8" width="17" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.85546875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
@@ -8943,7 +9003,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="273" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A273" s="4" t="s">
         <v>531</v>
       </c>
@@ -8954,7 +9014,7 @@
         <v>1035</v>
       </c>
     </row>
-    <row r="274" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A274" s="4" t="s">
         <v>59</v>
       </c>
@@ -8964,8 +9024,15 @@
       <c r="C274" s="4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="275" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="H274" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I274" s="3" t="str">
+        <f>VLOOKUP(H274,A:C,3,0)</f>
+        <v>TN0460</v>
+      </c>
+    </row>
+    <row r="275" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A275" s="4" t="s">
         <v>532</v>
       </c>
@@ -8976,7 +9043,7 @@
         <v>1036</v>
       </c>
     </row>
-    <row r="276" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A276" s="4" t="s">
         <v>295</v>
       </c>
@@ -8987,7 +9054,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="277" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A277" s="4" t="s">
         <v>533</v>
       </c>
@@ -8998,7 +9065,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="278" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A278" s="4" t="s">
         <v>534</v>
       </c>
@@ -9009,7 +9076,7 @@
         <v>1038</v>
       </c>
     </row>
-    <row r="279" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A279" s="4" t="s">
         <v>535</v>
       </c>
@@ -9020,7 +9087,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="280" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A280" s="4" t="s">
         <v>140</v>
       </c>
@@ -9031,7 +9098,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="281" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A281" s="4" t="s">
         <v>56</v>
       </c>
@@ -9042,7 +9109,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="282" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A282" s="4" t="s">
         <v>189</v>
       </c>
@@ -9053,7 +9120,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="283" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A283" s="4" t="s">
         <v>536</v>
       </c>
@@ -9064,7 +9131,7 @@
         <v>1040</v>
       </c>
     </row>
-    <row r="284" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A284" s="4" t="s">
         <v>537</v>
       </c>
@@ -9075,7 +9142,7 @@
         <v>1041</v>
       </c>
     </row>
-    <row r="285" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A285" s="4" t="s">
         <v>65</v>
       </c>
@@ -9086,7 +9153,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="286" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A286" s="4" t="s">
         <v>538</v>
       </c>
@@ -9097,7 +9164,7 @@
         <v>1042</v>
       </c>
     </row>
-    <row r="287" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A287" s="4" t="s">
         <v>539</v>
       </c>
@@ -9108,7 +9175,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="288" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:9" ht="15" x14ac:dyDescent="0.25">
       <c r="A288" s="4" t="s">
         <v>540</v>
       </c>
@@ -12714,6 +12781,138 @@
       </c>
       <c r="C615" s="5" t="s">
         <v>1324</v>
+      </c>
+    </row>
+    <row r="616" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A616" t="s">
+        <v>1832</v>
+      </c>
+      <c r="B616" t="s">
+        <v>141</v>
+      </c>
+      <c r="C616" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="617" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A617" t="s">
+        <v>1833</v>
+      </c>
+      <c r="B617" t="s">
+        <v>69</v>
+      </c>
+      <c r="C617" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="618" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A618" t="s">
+        <v>1811</v>
+      </c>
+      <c r="B618" t="s">
+        <v>1818</v>
+      </c>
+      <c r="C618" t="s">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="619" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A619" t="s">
+        <v>1812</v>
+      </c>
+      <c r="B619" t="s">
+        <v>1819</v>
+      </c>
+      <c r="C619" t="s">
+        <v>1826</v>
+      </c>
+    </row>
+    <row r="620" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A620" t="s">
+        <v>1813</v>
+      </c>
+      <c r="B620" t="s">
+        <v>1820</v>
+      </c>
+      <c r="C620" t="s">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="621" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A621" t="s">
+        <v>1814</v>
+      </c>
+      <c r="B621" t="s">
+        <v>1821</v>
+      </c>
+      <c r="C621" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="622" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A622" t="s">
+        <v>1815</v>
+      </c>
+      <c r="B622" t="s">
+        <v>1822</v>
+      </c>
+      <c r="C622" t="s">
+        <v>1829</v>
+      </c>
+    </row>
+    <row r="623" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A623" t="s">
+        <v>1816</v>
+      </c>
+      <c r="B623" t="s">
+        <v>1823</v>
+      </c>
+      <c r="C623" t="s">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="624" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A624" t="s">
+        <v>1817</v>
+      </c>
+      <c r="B624" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C624" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="625" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A625" t="s">
+        <v>301</v>
+      </c>
+      <c r="B625" t="s">
+        <v>302</v>
+      </c>
+      <c r="C625" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="626" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A626" t="s">
+        <v>269</v>
+      </c>
+      <c r="B626" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C626" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="627" spans="1:3" ht="15" x14ac:dyDescent="0.25">
+      <c r="A627" t="s">
+        <v>283</v>
+      </c>
+      <c r="B627" t="s">
+        <v>284</v>
+      </c>
+      <c r="C627" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>